<commit_message>
US 3.13: Updated component requirement and test case ids in test specification and test file.
</commit_message>
<xml_diff>
--- a/test/EnvironmentModel_Unit_Test_Specification_ EN.xlsx
+++ b/test/EnvironmentModel_Unit_Test_Specification_ EN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kumar\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{721919F5-66AC-47BB-ADB6-620E2E2954AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9979F87-33F3-4DE1-A23D-57721D3A055D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F18DBF44-7993-45AE-B09F-62D48714D91E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{F18DBF44-7993-45AE-B09F-62D48714D91E}"/>
   </bookViews>
   <sheets>
     <sheet name="Component Description" sheetId="5" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="60">
   <si>
     <t>ID</t>
   </si>
@@ -91,12 +91,6 @@
   </si>
   <si>
     <t>Test result comment</t>
-  </si>
-  <si>
-    <t>TC_OD001</t>
-  </si>
-  <si>
-    <t>TC_OD002</t>
   </si>
   <si>
     <t>M4</t>
@@ -160,48 +154,6 @@
 Expected Result 2: flg_calc_xyz is set to 1, bbox updated with one entry, and class_ids_confidence stores detected class and confidence.</t>
   </si>
   <si>
-    <t>US_3.13</t>
-  </si>
-  <si>
-    <t>AC_3.13.1</t>
-  </si>
-  <si>
-    <t>AC_3.13.2</t>
-  </si>
-  <si>
-    <t>AC_3.13.3</t>
-  </si>
-  <si>
-    <t>AC_3.13.4</t>
-  </si>
-  <si>
-    <t>AC_3.13.5</t>
-  </si>
-  <si>
-    <t>AC_3.13.6</t>
-  </si>
-  <si>
-    <t>AC_3.13.7</t>
-  </si>
-  <si>
-    <t>AC_3.13.8</t>
-  </si>
-  <si>
-    <t>AC_3.13.9</t>
-  </si>
-  <si>
-    <t>AC_3.13.10</t>
-  </si>
-  <si>
-    <t>TC_OD003</t>
-  </si>
-  <si>
-    <t>TC_OD004</t>
-  </si>
-  <si>
-    <t>TC_OD005</t>
-  </si>
-  <si>
     <t>Precondition: EnvironmentModel node is initialized with default yaw value.
 Test Step: Call odom_callback() with an Odometry message representing a 90° yaw rotation.
 Expected Result: Node yaw is updated to approximately π/2 radians.</t>
@@ -235,13 +187,6 @@
 Expected result 5: depth_callback handles the exception and bbox is cleared after processing.</t>
   </si>
   <si>
-    <t>AC_3.13.3, AC_3.13.4, AC_3.13.5, AC_3.13.6, AC_3.13.9, AC_3.13.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AC_3.13.2, AC_3.13.3,  AC_3.13.4
-</t>
-  </si>
-  <si>
     <t>Surendrakumar Koganti</t>
   </si>
   <si>
@@ -254,6 +199,61 @@
   </si>
   <si>
     <t>Additionally verified the new frame "v2x_frame" in RViZ visualisation tool.</t>
+  </si>
+  <si>
+    <t>EM001</t>
+  </si>
+  <si>
+    <t>EM001.1</t>
+  </si>
+  <si>
+    <t>EM001.2</t>
+  </si>
+  <si>
+    <t>EM001.3</t>
+  </si>
+  <si>
+    <t>EM001.4</t>
+  </si>
+  <si>
+    <t>EM001.5</t>
+  </si>
+  <si>
+    <t>EM001.6</t>
+  </si>
+  <si>
+    <t>EM001.7</t>
+  </si>
+  <si>
+    <t>EM001.8</t>
+  </si>
+  <si>
+    <t>EM001.9</t>
+  </si>
+  <si>
+    <t>EM001.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EM001.2, EM001.3,  EM001.4
+</t>
+  </si>
+  <si>
+    <t>EM001.3, EM001.4, EM001.5, EM001.6, EM001.9, EM001.10</t>
+  </si>
+  <si>
+    <t>TC_EM001</t>
+  </si>
+  <si>
+    <t>TC_EM002</t>
+  </si>
+  <si>
+    <t>TC_EM003</t>
+  </si>
+  <si>
+    <t>TC_EM004</t>
+  </si>
+  <si>
+    <t>TC_EM005</t>
   </si>
 </sst>
 </file>
@@ -666,12 +666,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -718,186 +718,183 @@
     </row>
     <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1104,22 +1101,22 @@
     </row>
     <row r="2" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>11</v>
@@ -1127,22 +1124,22 @@
     </row>
     <row r="3" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>11</v>
@@ -1150,22 +1147,22 @@
     </row>
     <row r="4" spans="1:9" ht="150" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>11</v>
@@ -1173,22 +1170,22 @@
     </row>
     <row r="5" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>11</v>
@@ -1196,10 +1193,10 @@
     </row>
     <row r="6" spans="1:9" ht="210" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>54</v>
@@ -1208,10 +1205,10 @@
         <v>7</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>11</v>
@@ -1264,7 +1261,7 @@
     </row>
     <row r="22" spans="2:2" ht="60" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.25">

</xml_diff>